<commit_message>
Atualiza custos e indicadores da DOA
</commit_message>
<xml_diff>
--- a/dados/custos_indicadores.xlsx
+++ b/dados/custos_indicadores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://factofundacao-my.sharepoint.com/personal/katarina_lemos_facto_org_br/Documents/Área de Trabalho/my_codes/precificacao_doa/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{06238C4E-BBDD-4287-A41D-A1D766E44EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF1491FD-7AD2-4EE3-9A83-3FFDD53899B2}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{06238C4E-BBDD-4287-A41D-A1D766E44EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99571D42-E43F-41EF-BFED-A87BB83CC223}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{3260332E-0F91-4634-B5BE-37CAFC126351}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{3260332E-0F91-4634-B5BE-37CAFC126351}"/>
   </bookViews>
   <sheets>
     <sheet name="ICP" sheetId="1" r:id="rId1"/>
@@ -2910,6 +2910,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{840A9CD1-4073-4C0E-BD17-8AA10D639CAA}">
   <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="27.7109375" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -2936,7 +2941,7 @@
         <v>151</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2950,7 +2955,7 @@
         <v>152</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2964,7 +2969,7 @@
         <v>153</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -2978,7 +2983,7 @@
         <v>154</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -2992,7 +2997,7 @@
         <v>155</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3006,7 +3011,7 @@
         <v>156</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3020,7 +3025,7 @@
         <v>157</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3090,7 +3095,7 @@
         <v>162</v>
       </c>
       <c r="D13">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3104,7 +3109,7 @@
         <v>163</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3118,7 +3123,7 @@
         <v>164</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3132,7 +3137,7 @@
         <v>165</v>
       </c>
       <c r="D16">
-        <v>3</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3146,7 +3151,7 @@
         <v>166</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3160,7 +3165,7 @@
         <v>167</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3174,7 +3179,7 @@
         <v>168</v>
       </c>
       <c r="D19">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3188,7 +3193,7 @@
         <v>169</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3202,7 +3207,7 @@
         <v>170</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3216,7 +3221,7 @@
         <v>171</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3230,7 +3235,7 @@
         <v>172</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -3244,7 +3249,7 @@
         <v>173</v>
       </c>
       <c r="D24">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -3258,7 +3263,7 @@
         <v>174</v>
       </c>
       <c r="D25">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -3272,7 +3277,7 @@
         <v>175</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -3286,7 +3291,7 @@
         <v>176</v>
       </c>
       <c r="D27">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -3300,7 +3305,7 @@
         <v>177</v>
       </c>
       <c r="D28">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3314,7 +3319,7 @@
         <v>178</v>
       </c>
       <c r="D29">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -3328,7 +3333,7 @@
         <v>179</v>
       </c>
       <c r="D30">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3342,7 +3347,7 @@
         <v>180</v>
       </c>
       <c r="D31">
-        <v>1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -3356,7 +3361,7 @@
         <v>181</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -3370,7 +3375,7 @@
         <v>182</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -3384,7 +3389,7 @@
         <v>183</v>
       </c>
       <c r="D34">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3398,7 +3403,7 @@
         <v>184</v>
       </c>
       <c r="D35">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -3412,7 +3417,7 @@
         <v>185</v>
       </c>
       <c r="D36">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -3426,7 +3431,7 @@
         <v>186</v>
       </c>
       <c r="D37">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -3440,7 +3445,7 @@
         <v>187</v>
       </c>
       <c r="D38">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>